<commit_message>
Refine workflow screens and spreadsheet editing
</commit_message>
<xml_diff>
--- a/4.Emails/07.08.26-Payment Plans CC Report 070826_FLYWIRE.xlsx
+++ b/4.Emails/07.08.26-Payment Plans CC Report 070826_FLYWIRE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\AP\Payment Plan Reports 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Renfrew\Workflow\4.Emails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD8593C3-CC45-4292-9677-3C5DC655E8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A22371-DADA-4D5A-AB64-E0DE110401E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1C9FAC53-BDD4-4D8B-B713-051F970F8DFA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1C9FAC53-BDD4-4D8B-B713-051F970F8DFA}"/>
   </bookViews>
   <sheets>
     <sheet name="PaymentsDetailedReport20260708_" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">PaymentsDetailedReport20260708_!$A$1:$K$5</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -95,10 +108,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,8 +247,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-0.14999847407452621"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -417,6 +438,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -557,7 +584,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -600,8 +627,9 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -621,8 +649,12 @@
     <xf numFmtId="0" fontId="16" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="43" fontId="0" fillId="33" borderId="0" xfId="42" applyFont="1" applyFill="1"/>
+    <xf numFmtId="40" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -650,6 +682,7 @@
     <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Comma" xfId="42" builtinId="3"/>
     <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
@@ -996,21 +1029,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C0AFC6D-38F6-45C8-A9AC-95DB0590889C}">
-  <dimension ref="A1:K17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:S17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" customWidth="1"/>
+    <col min="1" max="1" width="29.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.109375" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" customWidth="1"/>
-    <col min="7" max="7" width="18.42578125" customWidth="1"/>
-    <col min="9" max="9" width="22.28515625" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" customWidth="1"/>
-    <col min="11" max="11" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" customWidth="1"/>
+    <col min="7" max="7" width="18.44140625" customWidth="1"/>
+    <col min="9" max="9" width="22.33203125" customWidth="1"/>
+    <col min="10" max="10" width="17.6640625" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" customWidth="1"/>
+    <col min="13" max="13" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="30.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1045,7 +1081,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1079,8 +1115,36 @@
       <c r="K2" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="M2" s="7">
+        <f>F2</f>
+        <v>3557.03</v>
+      </c>
+      <c r="N2" s="8" t="str">
+        <f>H2&amp;": "&amp;I2&amp;"- "&amp;J2</f>
+        <v>136522: Paige Laufer- David J Laufer</v>
+      </c>
+      <c r="O2" s="9" t="str">
+        <f>Q2&amp;R2</f>
+        <v>VS-8719</v>
+      </c>
+      <c r="P2" s="10" t="str">
+        <f>LEFT(S2,4)</f>
+        <v>Visa</v>
+      </c>
+      <c r="Q2" s="10" t="str">
+        <f>IF(P2="Visa","VS-",IF(P2="Mast","MC-",IF(P2="Disc","DIS-",IF(P2="amer","AMEX-"))))</f>
+        <v>VS-</v>
+      </c>
+      <c r="R2" s="10" t="str">
+        <f>RIGHT(S2,4)</f>
+        <v>8719</v>
+      </c>
+      <c r="S2" s="10" t="str">
+        <f>MID(C2,8,(LEN(C2)-5))</f>
+        <v>Visa - 8719</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1093,7 +1157,7 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1111,7 +1175,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>21</v>
       </c>
@@ -1126,7 +1190,7 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1139,7 +1203,7 @@
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1152,7 +1216,7 @@
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -1165,7 +1229,7 @@
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1178,7 +1242,7 @@
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -1191,7 +1255,7 @@
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1204,7 +1268,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1217,7 +1281,7 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1230,7 +1294,7 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1243,7 +1307,7 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1256,7 +1320,7 @@
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -1269,7 +1333,7 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>

</xml_diff>